<commit_message>
chore(testing): simpan sementara paket uji performa vs SPSS dan ekspor ulang output SPSS
Cadangan sementara; rencananya dihapus lagi setelah diamankan.
- testing/performance-spss: skrip, hasil, dan log uji performa Statify vs SPSS
- ekspor ulang xlsx SPSS untuk referensi MV dan RM, sintaks .sps dengan OUTPUT EXPORT aktif
- hasil run performa Univariate terbaru

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/glm-mv-reference/spss-output/mv1_satu_populasi.xlsx
+++ b/testing/glm-mv-reference/spss-output/mv1_satu_populasi.xlsx
@@ -1417,124 +1417,124 @@
   </cellXfs>
   <cellStyles count="119">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="style1790153123405" xfId="1"/>
-    <cellStyle name="style1790153123435" xfId="2"/>
-    <cellStyle name="style1790153123460" xfId="3"/>
-    <cellStyle name="style1790153123488" xfId="4"/>
-    <cellStyle name="style1790153123512" xfId="5"/>
-    <cellStyle name="style1790153123529" xfId="6"/>
-    <cellStyle name="style1790153123549" xfId="7"/>
-    <cellStyle name="style1790153123581" xfId="8"/>
-    <cellStyle name="style1790153123605" xfId="9"/>
-    <cellStyle name="style1790153123630" xfId="10"/>
-    <cellStyle name="style1790153123657" xfId="11"/>
-    <cellStyle name="style1790153123678" xfId="12"/>
-    <cellStyle name="style1790153123703" xfId="13"/>
-    <cellStyle name="style1790153123730" xfId="14"/>
-    <cellStyle name="style1790153123750" xfId="15"/>
-    <cellStyle name="style1790153123763" xfId="16"/>
-    <cellStyle name="style1790153123785" xfId="17"/>
-    <cellStyle name="style1790153123811" xfId="18"/>
-    <cellStyle name="style1790153123834" xfId="19"/>
-    <cellStyle name="style1790153123858" xfId="20"/>
-    <cellStyle name="style1790153123880" xfId="21"/>
-    <cellStyle name="style1790153123906" xfId="22"/>
-    <cellStyle name="style1790153123933" xfId="23"/>
-    <cellStyle name="style1790153123958" xfId="24"/>
-    <cellStyle name="style1790153123986" xfId="25"/>
-    <cellStyle name="style1790153124010" xfId="26"/>
-    <cellStyle name="style1790153124035" xfId="27"/>
-    <cellStyle name="style1790153124063" xfId="28"/>
-    <cellStyle name="style1790153124086" xfId="29"/>
-    <cellStyle name="style1790153124110" xfId="30"/>
-    <cellStyle name="style1790153124130" xfId="31"/>
-    <cellStyle name="style1790153124149" xfId="32"/>
-    <cellStyle name="style1790153124160" xfId="33"/>
-    <cellStyle name="style1790153124186" xfId="34"/>
-    <cellStyle name="style1790153124205" xfId="35"/>
-    <cellStyle name="style1790153124223" xfId="36"/>
-    <cellStyle name="style1790153124251" xfId="37"/>
-    <cellStyle name="style1790153124274" xfId="38"/>
-    <cellStyle name="style1790153124295" xfId="39"/>
-    <cellStyle name="style1790153124317" xfId="40"/>
-    <cellStyle name="style1790153124340" xfId="41"/>
-    <cellStyle name="style1790153124366" xfId="42"/>
-    <cellStyle name="style1790153124388" xfId="43"/>
-    <cellStyle name="style1790153124411" xfId="44"/>
-    <cellStyle name="style1790153124433" xfId="45"/>
-    <cellStyle name="style1790153124454" xfId="46"/>
-    <cellStyle name="style1790153124475" xfId="47"/>
-    <cellStyle name="style1790153124497" xfId="48"/>
-    <cellStyle name="style1790153124519" xfId="49"/>
-    <cellStyle name="style1790153124534" xfId="50"/>
-    <cellStyle name="style1790153124550" xfId="51"/>
-    <cellStyle name="style1790153124564" xfId="52"/>
-    <cellStyle name="style1790153124582" xfId="53"/>
-    <cellStyle name="style1790153124597" xfId="54"/>
-    <cellStyle name="style1790153124614" xfId="55"/>
-    <cellStyle name="style1790153124632" xfId="56"/>
-    <cellStyle name="style1790153124646" xfId="57"/>
-    <cellStyle name="style1790153124663" xfId="58"/>
-    <cellStyle name="style1790153124684" xfId="59"/>
-    <cellStyle name="style1790153124698" xfId="60"/>
-    <cellStyle name="style1790153124714" xfId="61"/>
-    <cellStyle name="style1790153124729" xfId="62"/>
-    <cellStyle name="style1790153124744" xfId="63"/>
-    <cellStyle name="style1790153124762" xfId="64"/>
-    <cellStyle name="style1790153124778" xfId="65"/>
-    <cellStyle name="style1790153124800" xfId="66"/>
-    <cellStyle name="style1790153124823" xfId="67"/>
-    <cellStyle name="style1790153124842" xfId="68"/>
-    <cellStyle name="style1790153124865" xfId="69"/>
-    <cellStyle name="style1790153124885" xfId="70"/>
-    <cellStyle name="style1790153124910" xfId="71"/>
-    <cellStyle name="style1790153124928" xfId="72"/>
-    <cellStyle name="style1790153124944" xfId="73"/>
-    <cellStyle name="style1790153124962" xfId="74"/>
-    <cellStyle name="style1790153124979" xfId="75"/>
-    <cellStyle name="style1790153124994" xfId="76"/>
-    <cellStyle name="style1790153125010" xfId="77"/>
-    <cellStyle name="style1790153125026" xfId="78"/>
-    <cellStyle name="style1790153125042" xfId="79"/>
-    <cellStyle name="style1790153125056" xfId="80"/>
-    <cellStyle name="style1790153125073" xfId="81"/>
-    <cellStyle name="style1790153125088" xfId="82"/>
-    <cellStyle name="style1790153125102" xfId="83"/>
-    <cellStyle name="style1790153125117" xfId="84"/>
-    <cellStyle name="style1790153125132" xfId="85"/>
-    <cellStyle name="style1790153125142" xfId="86"/>
-    <cellStyle name="style1790153125170" xfId="87"/>
-    <cellStyle name="style1790153125185" xfId="88"/>
-    <cellStyle name="style1790153125203" xfId="89"/>
-    <cellStyle name="style1790153125225" xfId="90"/>
-    <cellStyle name="style1790153125247" xfId="91"/>
-    <cellStyle name="style1790153125271" xfId="92"/>
-    <cellStyle name="style1790153125294" xfId="93"/>
-    <cellStyle name="style1790153125311" xfId="94"/>
-    <cellStyle name="style1790153125338" xfId="95"/>
-    <cellStyle name="style1790153125353" xfId="96"/>
-    <cellStyle name="style1790153125368" xfId="97"/>
-    <cellStyle name="style1790153125383" xfId="98"/>
-    <cellStyle name="style1790153125399" xfId="99"/>
-    <cellStyle name="style1790153125414" xfId="100"/>
-    <cellStyle name="style1790153125429" xfId="101"/>
-    <cellStyle name="style1790153125445" xfId="102"/>
-    <cellStyle name="style1790153125463" xfId="103"/>
-    <cellStyle name="style1790153125486" xfId="104"/>
-    <cellStyle name="style1790153125498" xfId="105"/>
-    <cellStyle name="style1790153125517" xfId="106"/>
-    <cellStyle name="style1790153125539" xfId="107"/>
-    <cellStyle name="style1790153125556" xfId="108"/>
-    <cellStyle name="style1790153125573" xfId="109"/>
-    <cellStyle name="style1790153125588" xfId="110"/>
-    <cellStyle name="style1790153125603" xfId="111"/>
-    <cellStyle name="style1790153125621" xfId="112"/>
-    <cellStyle name="style1790153125635" xfId="113"/>
-    <cellStyle name="style1790153125645" xfId="114"/>
-    <cellStyle name="style1790153125666" xfId="115"/>
-    <cellStyle name="style1790153125686" xfId="116"/>
-    <cellStyle name="style1790153125705" xfId="117"/>
-    <cellStyle name="style1790153125722" xfId="118"/>
+    <cellStyle name="style1791027100825" xfId="1"/>
+    <cellStyle name="style1791027100868" xfId="2"/>
+    <cellStyle name="style1791027100895" xfId="3"/>
+    <cellStyle name="style1791027100925" xfId="4"/>
+    <cellStyle name="style1791027100956" xfId="5"/>
+    <cellStyle name="style1791027100989" xfId="6"/>
+    <cellStyle name="style1791027101013" xfId="7"/>
+    <cellStyle name="style1791027101050" xfId="8"/>
+    <cellStyle name="style1791027101073" xfId="9"/>
+    <cellStyle name="style1791027101105" xfId="10"/>
+    <cellStyle name="style1791027101138" xfId="11"/>
+    <cellStyle name="style1791027101164" xfId="12"/>
+    <cellStyle name="style1791027101192" xfId="13"/>
+    <cellStyle name="style1791027101225" xfId="14"/>
+    <cellStyle name="style1791027101254" xfId="15"/>
+    <cellStyle name="style1791027101277" xfId="16"/>
+    <cellStyle name="style1791027101296" xfId="17"/>
+    <cellStyle name="style1791027101324" xfId="18"/>
+    <cellStyle name="style1791027101351" xfId="19"/>
+    <cellStyle name="style1791027101374" xfId="20"/>
+    <cellStyle name="style1791027101402" xfId="21"/>
+    <cellStyle name="style1791027101428" xfId="22"/>
+    <cellStyle name="style1791027101472" xfId="23"/>
+    <cellStyle name="style1791027101499" xfId="24"/>
+    <cellStyle name="style1791027101525" xfId="25"/>
+    <cellStyle name="style1791027101553" xfId="26"/>
+    <cellStyle name="style1791027101584" xfId="27"/>
+    <cellStyle name="style1791027101618" xfId="28"/>
+    <cellStyle name="style1791027101644" xfId="29"/>
+    <cellStyle name="style1791027101670" xfId="30"/>
+    <cellStyle name="style1791027101694" xfId="31"/>
+    <cellStyle name="style1791027101714" xfId="32"/>
+    <cellStyle name="style1791027101735" xfId="33"/>
+    <cellStyle name="style1791027101758" xfId="34"/>
+    <cellStyle name="style1791027101784" xfId="35"/>
+    <cellStyle name="style1791027101804" xfId="36"/>
+    <cellStyle name="style1791027101830" xfId="37"/>
+    <cellStyle name="style1791027101854" xfId="38"/>
+    <cellStyle name="style1791027101878" xfId="39"/>
+    <cellStyle name="style1791027101899" xfId="40"/>
+    <cellStyle name="style1791027101930" xfId="41"/>
+    <cellStyle name="style1791027101954" xfId="42"/>
+    <cellStyle name="style1791027101974" xfId="43"/>
+    <cellStyle name="style1791027102002" xfId="44"/>
+    <cellStyle name="style1791027102026" xfId="45"/>
+    <cellStyle name="style1791027102046" xfId="46"/>
+    <cellStyle name="style1791027102074" xfId="47"/>
+    <cellStyle name="style1791027102094" xfId="48"/>
+    <cellStyle name="style1791027102121" xfId="49"/>
+    <cellStyle name="style1791027102136" xfId="50"/>
+    <cellStyle name="style1791027102154" xfId="51"/>
+    <cellStyle name="style1791027102167" xfId="52"/>
+    <cellStyle name="style1791027102190" xfId="53"/>
+    <cellStyle name="style1791027102206" xfId="54"/>
+    <cellStyle name="style1791027102224" xfId="55"/>
+    <cellStyle name="style1791027102242" xfId="56"/>
+    <cellStyle name="style1791027102258" xfId="57"/>
+    <cellStyle name="style1791027102275" xfId="58"/>
+    <cellStyle name="style1791027102302" xfId="59"/>
+    <cellStyle name="style1791027102322" xfId="60"/>
+    <cellStyle name="style1791027102339" xfId="61"/>
+    <cellStyle name="style1791027102355" xfId="62"/>
+    <cellStyle name="style1791027102374" xfId="63"/>
+    <cellStyle name="style1791027102393" xfId="64"/>
+    <cellStyle name="style1791027102409" xfId="65"/>
+    <cellStyle name="style1791027102434" xfId="66"/>
+    <cellStyle name="style1791027102458" xfId="67"/>
+    <cellStyle name="style1791027102486" xfId="68"/>
+    <cellStyle name="style1791027102513" xfId="69"/>
+    <cellStyle name="style1791027102537" xfId="70"/>
+    <cellStyle name="style1791027102562" xfId="71"/>
+    <cellStyle name="style1791027102574" xfId="72"/>
+    <cellStyle name="style1791027102594" xfId="73"/>
+    <cellStyle name="style1791027102614" xfId="74"/>
+    <cellStyle name="style1791027102634" xfId="75"/>
+    <cellStyle name="style1791027102651" xfId="76"/>
+    <cellStyle name="style1791027102667" xfId="77"/>
+    <cellStyle name="style1791027102688" xfId="78"/>
+    <cellStyle name="style1791027102704" xfId="79"/>
+    <cellStyle name="style1791027102723" xfId="80"/>
+    <cellStyle name="style1791027102737" xfId="81"/>
+    <cellStyle name="style1791027102758" xfId="82"/>
+    <cellStyle name="style1791027102774" xfId="83"/>
+    <cellStyle name="style1791027102792" xfId="84"/>
+    <cellStyle name="style1791027102810" xfId="85"/>
+    <cellStyle name="style1791027102825" xfId="86"/>
+    <cellStyle name="style1791027102847" xfId="87"/>
+    <cellStyle name="style1791027102869" xfId="88"/>
+    <cellStyle name="style1791027102894" xfId="89"/>
+    <cellStyle name="style1791027102916" xfId="90"/>
+    <cellStyle name="style1791027102944" xfId="91"/>
+    <cellStyle name="style1791027102968" xfId="92"/>
+    <cellStyle name="style1791027102994" xfId="93"/>
+    <cellStyle name="style1791027103021" xfId="94"/>
+    <cellStyle name="style1791027103047" xfId="95"/>
+    <cellStyle name="style1791027103064" xfId="96"/>
+    <cellStyle name="style1791027103082" xfId="97"/>
+    <cellStyle name="style1791027103102" xfId="98"/>
+    <cellStyle name="style1791027103122" xfId="99"/>
+    <cellStyle name="style1791027103144" xfId="100"/>
+    <cellStyle name="style1791027103157" xfId="101"/>
+    <cellStyle name="style1791027103175" xfId="102"/>
+    <cellStyle name="style1791027103204" xfId="103"/>
+    <cellStyle name="style1791027103227" xfId="104"/>
+    <cellStyle name="style1791027103244" xfId="105"/>
+    <cellStyle name="style1791027103263" xfId="106"/>
+    <cellStyle name="style1791027103289" xfId="107"/>
+    <cellStyle name="style1791027103307" xfId="108"/>
+    <cellStyle name="style1791027103326" xfId="109"/>
+    <cellStyle name="style1791027103347" xfId="110"/>
+    <cellStyle name="style1791027103366" xfId="111"/>
+    <cellStyle name="style1791027103383" xfId="112"/>
+    <cellStyle name="style1791027103395" xfId="113"/>
+    <cellStyle name="style1791027103415" xfId="114"/>
+    <cellStyle name="style1791027103436" xfId="115"/>
+    <cellStyle name="style1791027103460" xfId="116"/>
+    <cellStyle name="style1791027103477" xfId="117"/>
+    <cellStyle name="style1791027103498" xfId="118"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1961,7 +1961,7 @@
       <c r="B22" s="8"/>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>23-SEP-2026 15:45:23</t>
+          <t>03-OCT-2026 18:31:40</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>00:00:00.00</t>
+          <t>00:00:00.02</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>00:00:00.01</t>
+          <t>00:00:00.00</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       <c r="B67" s="8"/>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>23-SEP-2026 15:45:23</t>
+          <t>03-OCT-2026 18:31:40</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C78" s="16" t="inlineStr">
         <is>
-          <t>00:00:00.00</t>
+          <t>00:00:00.02</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>00:00:00.01</t>
+          <t>00:00:00.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(testing): hapus cadangan sementara paket uji performa dan ekspor ulang SPSS
Membatalkan fe7deb6c. Isinya sudah diarsipkan di luar repo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing/glm-mv-reference/spss-output/mv1_satu_populasi.xlsx
+++ b/testing/glm-mv-reference/spss-output/mv1_satu_populasi.xlsx
@@ -1417,124 +1417,124 @@
   </cellXfs>
   <cellStyles count="119">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="style1791027100825" xfId="1"/>
-    <cellStyle name="style1791027100868" xfId="2"/>
-    <cellStyle name="style1791027100895" xfId="3"/>
-    <cellStyle name="style1791027100925" xfId="4"/>
-    <cellStyle name="style1791027100956" xfId="5"/>
-    <cellStyle name="style1791027100989" xfId="6"/>
-    <cellStyle name="style1791027101013" xfId="7"/>
-    <cellStyle name="style1791027101050" xfId="8"/>
-    <cellStyle name="style1791027101073" xfId="9"/>
-    <cellStyle name="style1791027101105" xfId="10"/>
-    <cellStyle name="style1791027101138" xfId="11"/>
-    <cellStyle name="style1791027101164" xfId="12"/>
-    <cellStyle name="style1791027101192" xfId="13"/>
-    <cellStyle name="style1791027101225" xfId="14"/>
-    <cellStyle name="style1791027101254" xfId="15"/>
-    <cellStyle name="style1791027101277" xfId="16"/>
-    <cellStyle name="style1791027101296" xfId="17"/>
-    <cellStyle name="style1791027101324" xfId="18"/>
-    <cellStyle name="style1791027101351" xfId="19"/>
-    <cellStyle name="style1791027101374" xfId="20"/>
-    <cellStyle name="style1791027101402" xfId="21"/>
-    <cellStyle name="style1791027101428" xfId="22"/>
-    <cellStyle name="style1791027101472" xfId="23"/>
-    <cellStyle name="style1791027101499" xfId="24"/>
-    <cellStyle name="style1791027101525" xfId="25"/>
-    <cellStyle name="style1791027101553" xfId="26"/>
-    <cellStyle name="style1791027101584" xfId="27"/>
-    <cellStyle name="style1791027101618" xfId="28"/>
-    <cellStyle name="style1791027101644" xfId="29"/>
-    <cellStyle name="style1791027101670" xfId="30"/>
-    <cellStyle name="style1791027101694" xfId="31"/>
-    <cellStyle name="style1791027101714" xfId="32"/>
-    <cellStyle name="style1791027101735" xfId="33"/>
-    <cellStyle name="style1791027101758" xfId="34"/>
-    <cellStyle name="style1791027101784" xfId="35"/>
-    <cellStyle name="style1791027101804" xfId="36"/>
-    <cellStyle name="style1791027101830" xfId="37"/>
-    <cellStyle name="style1791027101854" xfId="38"/>
-    <cellStyle name="style1791027101878" xfId="39"/>
-    <cellStyle name="style1791027101899" xfId="40"/>
-    <cellStyle name="style1791027101930" xfId="41"/>
-    <cellStyle name="style1791027101954" xfId="42"/>
-    <cellStyle name="style1791027101974" xfId="43"/>
-    <cellStyle name="style1791027102002" xfId="44"/>
-    <cellStyle name="style1791027102026" xfId="45"/>
-    <cellStyle name="style1791027102046" xfId="46"/>
-    <cellStyle name="style1791027102074" xfId="47"/>
-    <cellStyle name="style1791027102094" xfId="48"/>
-    <cellStyle name="style1791027102121" xfId="49"/>
-    <cellStyle name="style1791027102136" xfId="50"/>
-    <cellStyle name="style1791027102154" xfId="51"/>
-    <cellStyle name="style1791027102167" xfId="52"/>
-    <cellStyle name="style1791027102190" xfId="53"/>
-    <cellStyle name="style1791027102206" xfId="54"/>
-    <cellStyle name="style1791027102224" xfId="55"/>
-    <cellStyle name="style1791027102242" xfId="56"/>
-    <cellStyle name="style1791027102258" xfId="57"/>
-    <cellStyle name="style1791027102275" xfId="58"/>
-    <cellStyle name="style1791027102302" xfId="59"/>
-    <cellStyle name="style1791027102322" xfId="60"/>
-    <cellStyle name="style1791027102339" xfId="61"/>
-    <cellStyle name="style1791027102355" xfId="62"/>
-    <cellStyle name="style1791027102374" xfId="63"/>
-    <cellStyle name="style1791027102393" xfId="64"/>
-    <cellStyle name="style1791027102409" xfId="65"/>
-    <cellStyle name="style1791027102434" xfId="66"/>
-    <cellStyle name="style1791027102458" xfId="67"/>
-    <cellStyle name="style1791027102486" xfId="68"/>
-    <cellStyle name="style1791027102513" xfId="69"/>
-    <cellStyle name="style1791027102537" xfId="70"/>
-    <cellStyle name="style1791027102562" xfId="71"/>
-    <cellStyle name="style1791027102574" xfId="72"/>
-    <cellStyle name="style1791027102594" xfId="73"/>
-    <cellStyle name="style1791027102614" xfId="74"/>
-    <cellStyle name="style1791027102634" xfId="75"/>
-    <cellStyle name="style1791027102651" xfId="76"/>
-    <cellStyle name="style1791027102667" xfId="77"/>
-    <cellStyle name="style1791027102688" xfId="78"/>
-    <cellStyle name="style1791027102704" xfId="79"/>
-    <cellStyle name="style1791027102723" xfId="80"/>
-    <cellStyle name="style1791027102737" xfId="81"/>
-    <cellStyle name="style1791027102758" xfId="82"/>
-    <cellStyle name="style1791027102774" xfId="83"/>
-    <cellStyle name="style1791027102792" xfId="84"/>
-    <cellStyle name="style1791027102810" xfId="85"/>
-    <cellStyle name="style1791027102825" xfId="86"/>
-    <cellStyle name="style1791027102847" xfId="87"/>
-    <cellStyle name="style1791027102869" xfId="88"/>
-    <cellStyle name="style1791027102894" xfId="89"/>
-    <cellStyle name="style1791027102916" xfId="90"/>
-    <cellStyle name="style1791027102944" xfId="91"/>
-    <cellStyle name="style1791027102968" xfId="92"/>
-    <cellStyle name="style1791027102994" xfId="93"/>
-    <cellStyle name="style1791027103021" xfId="94"/>
-    <cellStyle name="style1791027103047" xfId="95"/>
-    <cellStyle name="style1791027103064" xfId="96"/>
-    <cellStyle name="style1791027103082" xfId="97"/>
-    <cellStyle name="style1791027103102" xfId="98"/>
-    <cellStyle name="style1791027103122" xfId="99"/>
-    <cellStyle name="style1791027103144" xfId="100"/>
-    <cellStyle name="style1791027103157" xfId="101"/>
-    <cellStyle name="style1791027103175" xfId="102"/>
-    <cellStyle name="style1791027103204" xfId="103"/>
-    <cellStyle name="style1791027103227" xfId="104"/>
-    <cellStyle name="style1791027103244" xfId="105"/>
-    <cellStyle name="style1791027103263" xfId="106"/>
-    <cellStyle name="style1791027103289" xfId="107"/>
-    <cellStyle name="style1791027103307" xfId="108"/>
-    <cellStyle name="style1791027103326" xfId="109"/>
-    <cellStyle name="style1791027103347" xfId="110"/>
-    <cellStyle name="style1791027103366" xfId="111"/>
-    <cellStyle name="style1791027103383" xfId="112"/>
-    <cellStyle name="style1791027103395" xfId="113"/>
-    <cellStyle name="style1791027103415" xfId="114"/>
-    <cellStyle name="style1791027103436" xfId="115"/>
-    <cellStyle name="style1791027103460" xfId="116"/>
-    <cellStyle name="style1791027103477" xfId="117"/>
-    <cellStyle name="style1791027103498" xfId="118"/>
+    <cellStyle name="style1790153123405" xfId="1"/>
+    <cellStyle name="style1790153123435" xfId="2"/>
+    <cellStyle name="style1790153123460" xfId="3"/>
+    <cellStyle name="style1790153123488" xfId="4"/>
+    <cellStyle name="style1790153123512" xfId="5"/>
+    <cellStyle name="style1790153123529" xfId="6"/>
+    <cellStyle name="style1790153123549" xfId="7"/>
+    <cellStyle name="style1790153123581" xfId="8"/>
+    <cellStyle name="style1790153123605" xfId="9"/>
+    <cellStyle name="style1790153123630" xfId="10"/>
+    <cellStyle name="style1790153123657" xfId="11"/>
+    <cellStyle name="style1790153123678" xfId="12"/>
+    <cellStyle name="style1790153123703" xfId="13"/>
+    <cellStyle name="style1790153123730" xfId="14"/>
+    <cellStyle name="style1790153123750" xfId="15"/>
+    <cellStyle name="style1790153123763" xfId="16"/>
+    <cellStyle name="style1790153123785" xfId="17"/>
+    <cellStyle name="style1790153123811" xfId="18"/>
+    <cellStyle name="style1790153123834" xfId="19"/>
+    <cellStyle name="style1790153123858" xfId="20"/>
+    <cellStyle name="style1790153123880" xfId="21"/>
+    <cellStyle name="style1790153123906" xfId="22"/>
+    <cellStyle name="style1790153123933" xfId="23"/>
+    <cellStyle name="style1790153123958" xfId="24"/>
+    <cellStyle name="style1790153123986" xfId="25"/>
+    <cellStyle name="style1790153124010" xfId="26"/>
+    <cellStyle name="style1790153124035" xfId="27"/>
+    <cellStyle name="style1790153124063" xfId="28"/>
+    <cellStyle name="style1790153124086" xfId="29"/>
+    <cellStyle name="style1790153124110" xfId="30"/>
+    <cellStyle name="style1790153124130" xfId="31"/>
+    <cellStyle name="style1790153124149" xfId="32"/>
+    <cellStyle name="style1790153124160" xfId="33"/>
+    <cellStyle name="style1790153124186" xfId="34"/>
+    <cellStyle name="style1790153124205" xfId="35"/>
+    <cellStyle name="style1790153124223" xfId="36"/>
+    <cellStyle name="style1790153124251" xfId="37"/>
+    <cellStyle name="style1790153124274" xfId="38"/>
+    <cellStyle name="style1790153124295" xfId="39"/>
+    <cellStyle name="style1790153124317" xfId="40"/>
+    <cellStyle name="style1790153124340" xfId="41"/>
+    <cellStyle name="style1790153124366" xfId="42"/>
+    <cellStyle name="style1790153124388" xfId="43"/>
+    <cellStyle name="style1790153124411" xfId="44"/>
+    <cellStyle name="style1790153124433" xfId="45"/>
+    <cellStyle name="style1790153124454" xfId="46"/>
+    <cellStyle name="style1790153124475" xfId="47"/>
+    <cellStyle name="style1790153124497" xfId="48"/>
+    <cellStyle name="style1790153124519" xfId="49"/>
+    <cellStyle name="style1790153124534" xfId="50"/>
+    <cellStyle name="style1790153124550" xfId="51"/>
+    <cellStyle name="style1790153124564" xfId="52"/>
+    <cellStyle name="style1790153124582" xfId="53"/>
+    <cellStyle name="style1790153124597" xfId="54"/>
+    <cellStyle name="style1790153124614" xfId="55"/>
+    <cellStyle name="style1790153124632" xfId="56"/>
+    <cellStyle name="style1790153124646" xfId="57"/>
+    <cellStyle name="style1790153124663" xfId="58"/>
+    <cellStyle name="style1790153124684" xfId="59"/>
+    <cellStyle name="style1790153124698" xfId="60"/>
+    <cellStyle name="style1790153124714" xfId="61"/>
+    <cellStyle name="style1790153124729" xfId="62"/>
+    <cellStyle name="style1790153124744" xfId="63"/>
+    <cellStyle name="style1790153124762" xfId="64"/>
+    <cellStyle name="style1790153124778" xfId="65"/>
+    <cellStyle name="style1790153124800" xfId="66"/>
+    <cellStyle name="style1790153124823" xfId="67"/>
+    <cellStyle name="style1790153124842" xfId="68"/>
+    <cellStyle name="style1790153124865" xfId="69"/>
+    <cellStyle name="style1790153124885" xfId="70"/>
+    <cellStyle name="style1790153124910" xfId="71"/>
+    <cellStyle name="style1790153124928" xfId="72"/>
+    <cellStyle name="style1790153124944" xfId="73"/>
+    <cellStyle name="style1790153124962" xfId="74"/>
+    <cellStyle name="style1790153124979" xfId="75"/>
+    <cellStyle name="style1790153124994" xfId="76"/>
+    <cellStyle name="style1790153125010" xfId="77"/>
+    <cellStyle name="style1790153125026" xfId="78"/>
+    <cellStyle name="style1790153125042" xfId="79"/>
+    <cellStyle name="style1790153125056" xfId="80"/>
+    <cellStyle name="style1790153125073" xfId="81"/>
+    <cellStyle name="style1790153125088" xfId="82"/>
+    <cellStyle name="style1790153125102" xfId="83"/>
+    <cellStyle name="style1790153125117" xfId="84"/>
+    <cellStyle name="style1790153125132" xfId="85"/>
+    <cellStyle name="style1790153125142" xfId="86"/>
+    <cellStyle name="style1790153125170" xfId="87"/>
+    <cellStyle name="style1790153125185" xfId="88"/>
+    <cellStyle name="style1790153125203" xfId="89"/>
+    <cellStyle name="style1790153125225" xfId="90"/>
+    <cellStyle name="style1790153125247" xfId="91"/>
+    <cellStyle name="style1790153125271" xfId="92"/>
+    <cellStyle name="style1790153125294" xfId="93"/>
+    <cellStyle name="style1790153125311" xfId="94"/>
+    <cellStyle name="style1790153125338" xfId="95"/>
+    <cellStyle name="style1790153125353" xfId="96"/>
+    <cellStyle name="style1790153125368" xfId="97"/>
+    <cellStyle name="style1790153125383" xfId="98"/>
+    <cellStyle name="style1790153125399" xfId="99"/>
+    <cellStyle name="style1790153125414" xfId="100"/>
+    <cellStyle name="style1790153125429" xfId="101"/>
+    <cellStyle name="style1790153125445" xfId="102"/>
+    <cellStyle name="style1790153125463" xfId="103"/>
+    <cellStyle name="style1790153125486" xfId="104"/>
+    <cellStyle name="style1790153125498" xfId="105"/>
+    <cellStyle name="style1790153125517" xfId="106"/>
+    <cellStyle name="style1790153125539" xfId="107"/>
+    <cellStyle name="style1790153125556" xfId="108"/>
+    <cellStyle name="style1790153125573" xfId="109"/>
+    <cellStyle name="style1790153125588" xfId="110"/>
+    <cellStyle name="style1790153125603" xfId="111"/>
+    <cellStyle name="style1790153125621" xfId="112"/>
+    <cellStyle name="style1790153125635" xfId="113"/>
+    <cellStyle name="style1790153125645" xfId="114"/>
+    <cellStyle name="style1790153125666" xfId="115"/>
+    <cellStyle name="style1790153125686" xfId="116"/>
+    <cellStyle name="style1790153125705" xfId="117"/>
+    <cellStyle name="style1790153125722" xfId="118"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1961,7 +1961,7 @@
       <c r="B22" s="8"/>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>03-OCT-2026 18:31:40</t>
+          <t>23-SEP-2026 15:45:23</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>00:00:00.02</t>
+          <t>00:00:00.00</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>00:00:00.00</t>
+          <t>00:00:00.01</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       <c r="B67" s="8"/>
       <c r="C67" s="13" t="inlineStr">
         <is>
-          <t>03-OCT-2026 18:31:40</t>
+          <t>23-SEP-2026 15:45:23</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C78" s="16" t="inlineStr">
         <is>
-          <t>00:00:00.02</t>
+          <t>00:00:00.00</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>00:00:00.00</t>
+          <t>00:00:00.01</t>
         </is>
       </c>
     </row>

</xml_diff>